<commit_message>
some BTS improvements + added credits
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1326C960-0DED-4876-AA50-57AB78320786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{233893E5-285A-4DB0-8ACB-40E412CD4702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="204">
   <si>
     <t>ID</t>
   </si>
@@ -631,6 +631,12 @@
   </si>
   <si>
     <t>The 0.1%</t>
+  </si>
+  <si>
+    <t>Money doesn't buy happiness</t>
+  </si>
+  <si>
+    <t>Have over $100,000,000 with under 10 Joy</t>
   </si>
 </sst>
 </file>
@@ -966,7 +972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.44140625" customWidth="1"/>
@@ -2495,6 +2501,22 @@
       </c>
       <c r="F93" s="2"/>
     </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" s="2">
+        <v>92</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D94" s="2"/>
+      <c r="E94" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F94" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
backup before i do something drastic
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1231C7C9-C57D-49EF-9D94-3B919DBAEDAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616F12AF-0D8B-4C3A-9DD8-947B239EC815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="230">
   <si>
     <t>ID</t>
   </si>
@@ -108,9 +108,6 @@
     <t>Reward (if applicable)</t>
   </si>
   <si>
-    <t>Wait I get something for this right?</t>
-  </si>
-  <si>
     <t>Get 10 achievements</t>
   </si>
   <si>
@@ -120,12 +117,6 @@
     <t>Achieve all perfect stats</t>
   </si>
   <si>
-    <t>Old</t>
-  </si>
-  <si>
-    <t>Reach 80 years old</t>
-  </si>
-  <si>
     <t>Bed Tundy</t>
   </si>
   <si>
@@ -189,9 +180,6 @@
     <t>Have both 100 Karma and 100 Evality at the same time</t>
   </si>
   <si>
-    <t>Very responsible with my money</t>
-  </si>
-  <si>
     <t>Be $100,000 in debt</t>
   </si>
   <si>
@@ -576,9 +564,6 @@
     <t>Have an intellect of 0 and 100 joy</t>
   </si>
   <si>
-    <t>Dunning-Kruger effect</t>
-  </si>
-  <si>
     <t>Die by electrocution</t>
   </si>
   <si>
@@ -612,9 +597,6 @@
     <t>Be a gay man</t>
   </si>
   <si>
-    <t>Yeah, well, we're all jealous of you</t>
-  </si>
-  <si>
     <t>Onion</t>
   </si>
   <si>
@@ -679,6 +661,60 @@
   </si>
   <si>
     <t>Be 99 years old and have 99 joy, 99 health, 99 intellect, 99 looks, 99 relationship with 99 people, and $99.</t>
+  </si>
+  <si>
+    <t>Go from having an evality of 100 to 0 in the same life</t>
+  </si>
+  <si>
+    <t>Change</t>
+  </si>
+  <si>
+    <t>Polarising</t>
+  </si>
+  <si>
+    <t>Have a relationship of -100 with one person and 100 with another at the same time</t>
+  </si>
+  <si>
+    <t>Happy</t>
+  </si>
+  <si>
+    <t>Die with 0 evality</t>
+  </si>
+  <si>
+    <t>Everything is fine.</t>
+  </si>
+  <si>
+    <t>Ignorance is bliss</t>
+  </si>
+  <si>
+    <t>Very responsible with money</t>
+  </si>
+  <si>
+    <t>Wait I get something for these right?</t>
+  </si>
+  <si>
+    <t>Indie hit</t>
+  </si>
+  <si>
+    <t>Make a video game by yourself that generates over $1,000,000 in revenue</t>
+  </si>
+  <si>
+    <t>Make a board game</t>
+  </si>
+  <si>
+    <t>More like bored game</t>
+  </si>
+  <si>
+    <t>Eventful</t>
+  </si>
+  <si>
+    <t>Encounter one event every year for 20 consecutive years</t>
+  </si>
+  <si>
+    <t>This achievement will sunset in 30 days</t>
+  </si>
+  <si>
+    <t>Discontinue a product</t>
   </si>
 </sst>
 </file>
@@ -1014,7 +1050,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.44140625" customWidth="1"/>
@@ -1038,7 +1074,7 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>26</v>
@@ -1052,7 +1088,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>5</v>
@@ -1070,7 +1106,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="3" t="s">
@@ -1182,7 +1218,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="3" t="s">
@@ -1211,17 +1247,17 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="3" t="s">
         <v>18</v>
       </c>
       <c r="F12" s="4">
-        <v>1000</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1229,14 +1265,14 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>31</v>
+        <v>222</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>32</v>
+        <v>223</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="3" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F13" s="2"/>
     </row>
@@ -1245,10 +1281,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="3" t="s">
@@ -1261,10 +1297,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="3" t="s">
@@ -1277,10 +1313,10 @@
         <v>14</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="3" t="s">
@@ -1293,14 +1329,14 @@
         <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F17" s="2"/>
     </row>
@@ -1309,10 +1345,10 @@
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="3" t="s">
@@ -1327,10 +1363,10 @@
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="3" t="s">
@@ -1343,10 +1379,10 @@
         <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="3" t="s">
@@ -1361,10 +1397,10 @@
         <v>19</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="3" t="s">
@@ -1377,14 +1413,14 @@
         <v>20</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F22" s="2"/>
     </row>
@@ -1393,14 +1429,14 @@
         <v>21</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F23" s="2"/>
     </row>
@@ -1409,10 +1445,10 @@
         <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>54</v>
+        <v>220</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="3" t="s">
@@ -1425,10 +1461,10 @@
         <v>23</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="3" t="s">
@@ -1443,14 +1479,14 @@
         <v>24</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F26" s="2"/>
     </row>
@@ -1459,10 +1495,10 @@
         <v>25</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="3" t="s">
@@ -1475,10 +1511,10 @@
         <v>26</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="3" t="s">
@@ -1491,14 +1527,14 @@
         <v>27</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F29" s="2"/>
     </row>
@@ -1507,10 +1543,10 @@
         <v>28</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="3" t="s">
@@ -1525,10 +1561,10 @@
         <v>29</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="3" t="s">
@@ -1541,14 +1577,14 @@
         <v>30</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="3" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F32" s="4">
         <v>1000000</v>
@@ -1559,10 +1595,10 @@
         <v>31</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="3" t="s">
@@ -1575,10 +1611,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="3" t="s">
@@ -1591,14 +1627,14 @@
         <v>33</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F35" s="2"/>
     </row>
@@ -1607,10 +1643,10 @@
         <v>34</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="3" t="s">
@@ -1623,10 +1659,10 @@
         <v>35</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="3" t="s">
@@ -1639,10 +1675,10 @@
         <v>36</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="3" t="s">
@@ -1655,14 +1691,14 @@
         <v>37</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F39" s="2"/>
     </row>
@@ -1671,10 +1707,10 @@
         <v>38</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="3" t="s">
@@ -1687,14 +1723,14 @@
         <v>39</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F41" s="4">
         <v>10000</v>
@@ -1705,14 +1741,14 @@
         <v>40</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F42" s="2"/>
     </row>
@@ -1721,14 +1757,14 @@
         <v>41</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F43" s="4">
         <v>50000</v>
@@ -1739,10 +1775,10 @@
         <v>42</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="3" t="s">
@@ -1757,10 +1793,10 @@
         <v>43</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="3" t="s">
@@ -1773,10 +1809,10 @@
         <v>44</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="3" t="s">
@@ -1789,10 +1825,10 @@
         <v>45</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="3" t="s">
@@ -1805,10 +1841,10 @@
         <v>46</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="3" t="s">
@@ -1821,13 +1857,13 @@
         <v>47</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>12</v>
@@ -1839,13 +1875,13 @@
         <v>48</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>12</v>
@@ -1857,16 +1893,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F51" s="2"/>
     </row>
@@ -1875,10 +1911,10 @@
         <v>50</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="3" t="s">
@@ -1891,10 +1927,10 @@
         <v>51</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="3" t="s">
@@ -1907,10 +1943,10 @@
         <v>52</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="3" t="s">
@@ -1923,10 +1959,10 @@
         <v>53</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="3" t="s">
@@ -1939,10 +1975,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="3" t="s">
@@ -1955,10 +1991,10 @@
         <v>55</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="3" t="s">
@@ -1971,10 +2007,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="3" t="s">
@@ -1987,10 +2023,10 @@
         <v>57</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="3" t="s">
@@ -2003,10 +2039,10 @@
         <v>58</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="3" t="s">
@@ -2018,10 +2054,10 @@
         <v>59</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="3" t="s">
@@ -2034,10 +2070,10 @@
         <v>60</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="3" t="s">
@@ -2049,10 +2085,10 @@
         <v>61</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="3" t="s">
@@ -2065,13 +2101,13 @@
         <v>62</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>12</v>
@@ -2085,10 +2121,10 @@
         <v>63</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="3" t="s">
@@ -2101,10 +2137,10 @@
         <v>64</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="3" t="s">
@@ -2117,10 +2153,10 @@
         <v>65</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="3" t="s">
@@ -2133,10 +2169,10 @@
         <v>66</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D68" s="2"/>
       <c r="E68" s="3" t="s">
@@ -2149,10 +2185,10 @@
         <v>67</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D69" s="2"/>
       <c r="E69" s="3" t="s">
@@ -2167,10 +2203,10 @@
         <v>68</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D70" s="2"/>
       <c r="E70" s="3" t="s">
@@ -2183,14 +2219,14 @@
         <v>69</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D71" s="2"/>
       <c r="E71" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F71" s="2"/>
     </row>
@@ -2199,10 +2235,10 @@
         <v>70</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D72" s="2"/>
       <c r="E72" s="3" t="s">
@@ -2215,10 +2251,10 @@
         <v>71</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D73" s="2"/>
       <c r="E73" s="3" t="s">
@@ -2231,10 +2267,10 @@
         <v>72</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D74" s="2"/>
       <c r="E74" s="3" t="s">
@@ -2247,10 +2283,10 @@
         <v>73</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D75" s="2"/>
       <c r="E75" s="3" t="s">
@@ -2263,14 +2299,14 @@
         <v>74</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D76" s="2"/>
       <c r="E76" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F76" s="2"/>
     </row>
@@ -2279,10 +2315,10 @@
         <v>75</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D77" s="2"/>
       <c r="E77" s="3" t="s">
@@ -2295,10 +2331,10 @@
         <v>76</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D78" s="2"/>
       <c r="E78" s="3" t="s">
@@ -2311,16 +2347,16 @@
         <v>77</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="E79" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F79" s="2"/>
     </row>
@@ -2329,10 +2365,10 @@
         <v>78</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D80" s="3"/>
       <c r="E80" s="3" t="s">
@@ -2345,14 +2381,14 @@
         <v>79</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F81" s="2"/>
     </row>
@@ -2361,10 +2397,10 @@
         <v>80</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D82" s="2"/>
       <c r="E82" s="3" t="s">
@@ -2377,10 +2413,10 @@
         <v>81</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D83" s="2"/>
       <c r="E83" s="3" t="s">
@@ -2393,10 +2429,10 @@
         <v>82</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>12</v>
@@ -2407,10 +2443,10 @@
         <v>83</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D85" s="2"/>
       <c r="E85" s="3" t="s">
@@ -2423,10 +2459,10 @@
         <v>84</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D86" s="2"/>
       <c r="E86" s="3" t="s">
@@ -2439,14 +2475,14 @@
         <v>85</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F87" s="2"/>
     </row>
@@ -2455,10 +2491,10 @@
         <v>86</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>183</v>
+        <v>219</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D88" s="2"/>
       <c r="E88" s="3" t="s">
@@ -2471,10 +2507,10 @@
         <v>87</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D89" s="2"/>
       <c r="E89" s="3" t="s">
@@ -2487,10 +2523,10 @@
         <v>88</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="3" t="s">
@@ -2502,10 +2538,10 @@
         <v>89</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D91" s="2"/>
       <c r="E91" s="3" t="s">
@@ -2518,10 +2554,10 @@
         <v>90</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>12</v>
@@ -2532,10 +2568,10 @@
         <v>91</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="D93" s="2"/>
       <c r="E93" s="3" t="s">
@@ -2548,10 +2584,10 @@
         <v>92</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D94" s="2"/>
       <c r="E94" s="3" t="s">
@@ -2564,10 +2600,10 @@
         <v>93</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D95" s="2"/>
       <c r="E95" s="3" t="s">
@@ -2580,10 +2616,10 @@
         <v>94</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="D96" s="2"/>
       <c r="E96" s="3" t="s">
@@ -2596,10 +2632,10 @@
         <v>95</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="D97" s="2"/>
       <c r="E97" s="3" t="s">
@@ -2612,10 +2648,10 @@
         <v>96</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="D98" s="2"/>
       <c r="E98" s="3" t="s">
@@ -2628,14 +2664,14 @@
         <v>97</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D99" s="2"/>
       <c r="E99" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F99" s="2"/>
     </row>
@@ -2644,10 +2680,10 @@
         <v>98</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D100" s="2"/>
       <c r="E100" s="3" t="s">
@@ -2660,16 +2696,110 @@
         <v>99</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D101" s="2"/>
       <c r="E101" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F101" s="2"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="2">
+        <v>100</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="D102" s="2"/>
+      <c r="E102" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F102" s="2"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="2">
+        <v>101</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D103" s="2"/>
+      <c r="E103" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F103" s="2"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="2">
+        <v>102</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="D104" s="2"/>
+      <c r="E104" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F104" s="2"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="2">
+        <v>103</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="D105" s="2"/>
+      <c r="E105" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F105" s="2"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="2">
+        <v>104</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" s="2">
+        <v>105</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D107" s="2"/>
+      <c r="E107" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F107" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
working life saving on demand!!
in settings -> save game
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616F12AF-0D8B-4C3A-9DD8-947B239EC815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690EE796-4C04-41C3-BD62-9932B13E98C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,9 +210,6 @@
     <t>Do a Kennedy</t>
   </si>
   <si>
-    <t>Inception more like contraception</t>
-  </si>
-  <si>
     <t>Make Bad Life Simulator</t>
   </si>
   <si>
@@ -715,6 +712,9 @@
   </si>
   <si>
     <t>Discontinue a product</t>
+  </si>
+  <si>
+    <t>Mitosis</t>
   </si>
 </sst>
 </file>
@@ -1074,7 +1074,7 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>26</v>
@@ -1218,7 +1218,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="3" t="s">
@@ -1247,7 +1247,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>27</v>
@@ -1265,10 +1265,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>222</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>223</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="3" t="s">
@@ -1429,7 +1429,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>50</v>
@@ -1445,7 +1445,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>51</v>
@@ -1464,7 +1464,7 @@
         <v>52</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="3" t="s">
@@ -1543,10 +1543,10 @@
         <v>28</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="3" t="s">
@@ -1561,10 +1561,10 @@
         <v>29</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="3" t="s">
@@ -1577,14 +1577,14 @@
         <v>30</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>186</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>187</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F32" s="4">
         <v>1000000</v>
@@ -1595,10 +1595,10 @@
         <v>31</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="3" t="s">
@@ -1611,10 +1611,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="3" t="s">
@@ -1627,10 +1627,10 @@
         <v>33</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>69</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="3" t="s">
@@ -1643,10 +1643,10 @@
         <v>34</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="3" t="s">
@@ -1659,10 +1659,10 @@
         <v>35</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="3" t="s">
@@ -1675,10 +1675,10 @@
         <v>36</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="3" t="s">
@@ -1691,10 +1691,10 @@
         <v>37</v>
       </c>
       <c r="B39" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>77</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="3" t="s">
@@ -1707,10 +1707,10 @@
         <v>38</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="3" t="s">
@@ -1723,10 +1723,10 @@
         <v>39</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="3" t="s">
@@ -1741,10 +1741,10 @@
         <v>40</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="3" t="s">
@@ -1757,10 +1757,10 @@
         <v>41</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="3" t="s">
@@ -1775,10 +1775,10 @@
         <v>42</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="3" t="s">
@@ -1793,10 +1793,10 @@
         <v>43</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>88</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="3" t="s">
@@ -1809,10 +1809,10 @@
         <v>44</v>
       </c>
       <c r="B46" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C46" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>90</v>
       </c>
       <c r="D46" s="2"/>
       <c r="E46" s="3" t="s">
@@ -1825,10 +1825,10 @@
         <v>45</v>
       </c>
       <c r="B47" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" s="3" t="s">
         <v>91</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>92</v>
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="3" t="s">
@@ -1844,7 +1844,7 @@
         <v>41</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="3" t="s">
@@ -1857,13 +1857,13 @@
         <v>47</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C49" s="3" t="s">
+      <c r="D49" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>96</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>12</v>
@@ -1875,13 +1875,13 @@
         <v>48</v>
       </c>
       <c r="B50" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C50" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="D50" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>99</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>12</v>
@@ -1893,13 +1893,13 @@
         <v>49</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C51" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="D51" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>49</v>
@@ -1911,10 +1911,10 @@
         <v>50</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="3" t="s">
@@ -1927,10 +1927,10 @@
         <v>51</v>
       </c>
       <c r="B53" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="3" t="s">
@@ -1943,10 +1943,10 @@
         <v>52</v>
       </c>
       <c r="B54" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C54" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>106</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="3" t="s">
@@ -1959,10 +1959,10 @@
         <v>53</v>
       </c>
       <c r="B55" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C55" s="3" t="s">
         <v>108</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>109</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="3" t="s">
@@ -1975,10 +1975,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="3" t="s">
@@ -1991,10 +1991,10 @@
         <v>55</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="3" t="s">
@@ -2007,10 +2007,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>113</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="3" t="s">
@@ -2023,10 +2023,10 @@
         <v>57</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="3" t="s">
@@ -2039,10 +2039,10 @@
         <v>58</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="3" t="s">
@@ -2054,10 +2054,10 @@
         <v>59</v>
       </c>
       <c r="B61" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C61" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>119</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="3" t="s">
@@ -2070,10 +2070,10 @@
         <v>60</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="3" t="s">
@@ -2085,10 +2085,10 @@
         <v>61</v>
       </c>
       <c r="B63" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C63" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>122</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="3" t="s">
@@ -2101,13 +2101,13 @@
         <v>62</v>
       </c>
       <c r="B64" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="D64" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>12</v>
@@ -2121,10 +2121,10 @@
         <v>63</v>
       </c>
       <c r="B65" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C65" s="3" t="s">
         <v>127</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>128</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="3" t="s">
@@ -2137,10 +2137,10 @@
         <v>64</v>
       </c>
       <c r="B66" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C66" s="3" t="s">
         <v>129</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>130</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="3" t="s">
@@ -2153,10 +2153,10 @@
         <v>65</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C67" s="3" t="s">
         <v>131</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>132</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="3" t="s">
@@ -2169,10 +2169,10 @@
         <v>66</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D68" s="2"/>
       <c r="E68" s="3" t="s">
@@ -2185,10 +2185,10 @@
         <v>67</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D69" s="2"/>
       <c r="E69" s="3" t="s">
@@ -2203,10 +2203,10 @@
         <v>68</v>
       </c>
       <c r="B70" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C70" s="3" t="s">
         <v>136</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>137</v>
       </c>
       <c r="D70" s="2"/>
       <c r="E70" s="3" t="s">
@@ -2219,10 +2219,10 @@
         <v>69</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D71" s="2"/>
       <c r="E71" s="3" t="s">
@@ -2235,10 +2235,10 @@
         <v>70</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D72" s="2"/>
       <c r="E72" s="3" t="s">
@@ -2251,10 +2251,10 @@
         <v>71</v>
       </c>
       <c r="B73" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C73" s="3" t="s">
         <v>143</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>144</v>
       </c>
       <c r="D73" s="2"/>
       <c r="E73" s="3" t="s">
@@ -2267,10 +2267,10 @@
         <v>72</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D74" s="2"/>
       <c r="E74" s="3" t="s">
@@ -2283,10 +2283,10 @@
         <v>73</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D75" s="2"/>
       <c r="E75" s="3" t="s">
@@ -2299,10 +2299,10 @@
         <v>74</v>
       </c>
       <c r="B76" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C76" s="3" t="s">
         <v>148</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>149</v>
       </c>
       <c r="D76" s="2"/>
       <c r="E76" s="3" t="s">
@@ -2315,10 +2315,10 @@
         <v>75</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D77" s="2"/>
       <c r="E77" s="3" t="s">
@@ -2331,10 +2331,10 @@
         <v>76</v>
       </c>
       <c r="B78" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="C78" s="3" t="s">
         <v>152</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>153</v>
       </c>
       <c r="D78" s="2"/>
       <c r="E78" s="3" t="s">
@@ -2347,13 +2347,13 @@
         <v>77</v>
       </c>
       <c r="B79" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C79" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="D79" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>38</v>
@@ -2365,10 +2365,10 @@
         <v>78</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C80" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>160</v>
       </c>
       <c r="D80" s="3"/>
       <c r="E80" s="3" t="s">
@@ -2381,10 +2381,10 @@
         <v>79</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="3" t="s">
@@ -2397,10 +2397,10 @@
         <v>80</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D82" s="2"/>
       <c r="E82" s="3" t="s">
@@ -2413,10 +2413,10 @@
         <v>81</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D83" s="2"/>
       <c r="E83" s="3" t="s">
@@ -2429,10 +2429,10 @@
         <v>82</v>
       </c>
       <c r="B84" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C84" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>168</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>12</v>
@@ -2443,10 +2443,10 @@
         <v>83</v>
       </c>
       <c r="B85" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C85" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>170</v>
       </c>
       <c r="D85" s="2"/>
       <c r="E85" s="3" t="s">
@@ -2459,10 +2459,10 @@
         <v>84</v>
       </c>
       <c r="B86" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C86" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>174</v>
       </c>
       <c r="D86" s="2"/>
       <c r="E86" s="3" t="s">
@@ -2475,10 +2475,10 @@
         <v>85</v>
       </c>
       <c r="B87" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C87" s="3" t="s">
         <v>175</v>
-      </c>
-      <c r="C87" s="3" t="s">
-        <v>176</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="3" t="s">
@@ -2491,10 +2491,10 @@
         <v>86</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D88" s="2"/>
       <c r="E88" s="3" t="s">
@@ -2507,10 +2507,10 @@
         <v>87</v>
       </c>
       <c r="B89" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C89" s="3" t="s">
         <v>180</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>181</v>
       </c>
       <c r="D89" s="2"/>
       <c r="E89" s="3" t="s">
@@ -2523,10 +2523,10 @@
         <v>88</v>
       </c>
       <c r="B90" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C90" s="3" t="s">
         <v>182</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>183</v>
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="3" t="s">
@@ -2538,10 +2538,10 @@
         <v>89</v>
       </c>
       <c r="B91" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C91" s="3" t="s">
         <v>188</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>189</v>
       </c>
       <c r="D91" s="2"/>
       <c r="E91" s="3" t="s">
@@ -2554,10 +2554,10 @@
         <v>90</v>
       </c>
       <c r="B92" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C92" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>12</v>
@@ -2568,10 +2568,10 @@
         <v>91</v>
       </c>
       <c r="B93" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="C93" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="C93" s="3" t="s">
-        <v>193</v>
       </c>
       <c r="D93" s="2"/>
       <c r="E93" s="3" t="s">
@@ -2584,10 +2584,10 @@
         <v>92</v>
       </c>
       <c r="B94" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C94" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>197</v>
       </c>
       <c r="D94" s="2"/>
       <c r="E94" s="3" t="s">
@@ -2600,10 +2600,10 @@
         <v>93</v>
       </c>
       <c r="B95" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C95" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="C95" s="3" t="s">
-        <v>199</v>
       </c>
       <c r="D95" s="2"/>
       <c r="E95" s="3" t="s">
@@ -2616,10 +2616,10 @@
         <v>94</v>
       </c>
       <c r="B96" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C96" s="3" t="s">
         <v>200</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>201</v>
       </c>
       <c r="D96" s="2"/>
       <c r="E96" s="3" t="s">
@@ -2632,10 +2632,10 @@
         <v>95</v>
       </c>
       <c r="B97" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C97" s="3" t="s">
         <v>202</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>203</v>
       </c>
       <c r="D97" s="2"/>
       <c r="E97" s="3" t="s">
@@ -2648,10 +2648,10 @@
         <v>96</v>
       </c>
       <c r="B98" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="C98" s="3" t="s">
         <v>204</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>205</v>
       </c>
       <c r="D98" s="2"/>
       <c r="E98" s="3" t="s">
@@ -2664,10 +2664,10 @@
         <v>97</v>
       </c>
       <c r="B99" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C99" s="3" t="s">
         <v>206</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>207</v>
       </c>
       <c r="D99" s="2"/>
       <c r="E99" s="3" t="s">
@@ -2680,10 +2680,10 @@
         <v>98</v>
       </c>
       <c r="B100" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C100" s="3" t="s">
         <v>208</v>
-      </c>
-      <c r="C100" s="3" t="s">
-        <v>209</v>
       </c>
       <c r="D100" s="2"/>
       <c r="E100" s="3" t="s">
@@ -2696,10 +2696,10 @@
         <v>99</v>
       </c>
       <c r="B101" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="C101" s="3" t="s">
         <v>210</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>211</v>
       </c>
       <c r="D101" s="2"/>
       <c r="E101" s="3" t="s">
@@ -2712,10 +2712,10 @@
         <v>100</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D102" s="2"/>
       <c r="E102" s="3" t="s">
@@ -2728,10 +2728,10 @@
         <v>101</v>
       </c>
       <c r="B103" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C103" s="3" t="s">
         <v>214</v>
-      </c>
-      <c r="C103" s="3" t="s">
-        <v>215</v>
       </c>
       <c r="D103" s="2"/>
       <c r="E103" s="3" t="s">
@@ -2744,10 +2744,10 @@
         <v>102</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D104" s="2"/>
       <c r="E104" s="3" t="s">
@@ -2760,10 +2760,10 @@
         <v>103</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D105" s="2"/>
       <c r="E105" s="3" t="s">
@@ -2776,13 +2776,13 @@
         <v>104</v>
       </c>
       <c r="B106" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C106" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="C106" s="3" t="s">
-        <v>227</v>
-      </c>
       <c r="E106" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
@@ -2790,10 +2790,10 @@
         <v>105</v>
       </c>
       <c r="B107" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C107" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>229</v>
       </c>
       <c r="D107" s="2"/>
       <c r="E107" s="3" t="s">

</xml_diff>

<commit_message>
life save file buttons scrolling
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690EE796-4C04-41C3-BD62-9932B13E98C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03689733-3534-4286-BA19-C4D0F6364498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="240">
   <si>
     <t>ID</t>
   </si>
@@ -715,6 +715,36 @@
   </si>
   <si>
     <t>Mitosis</t>
+  </si>
+  <si>
+    <t>I can cino</t>
+  </si>
+  <si>
+    <t>Win a casino game</t>
+  </si>
+  <si>
+    <t>I can't cino</t>
+  </si>
+  <si>
+    <t>Lose a casino game</t>
+  </si>
+  <si>
+    <t>Ping</t>
+  </si>
+  <si>
+    <t>Pang</t>
+  </si>
+  <si>
+    <t>Beat the AI</t>
+  </si>
+  <si>
+    <t>Beat the AI at Pang</t>
+  </si>
+  <si>
+    <t>Get a score of 30 or over on Pang</t>
+  </si>
+  <si>
+    <t>Get a score of 50 or over on pang</t>
   </si>
 </sst>
 </file>
@@ -1050,7 +1080,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.44140625" customWidth="1"/>
@@ -2530,7 +2560,7 @@
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="3" t="s">
-        <v>18</v>
+        <v>184</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
@@ -2800,6 +2830,76 @@
         <v>7</v>
       </c>
       <c r="F107" s="2"/>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="2">
+        <v>106</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="2">
+        <v>107</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="2">
+        <v>108</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="2">
+        <v>109</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" s="2">
+        <v>110</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
wow, NOW all I need to do is add any funcitonality
Yes, this entire thing was JUST switching between load and delete mode in the save file manager. Don't talk to me about switching between load and delete mode in the save file manager.
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03689733-3534-4286-BA19-C4D0F6364498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E3A699-7CC9-4EA2-8B0D-DAA4B26B98E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2855,9 +2855,11 @@
       <c r="C109" s="3" t="s">
         <v>233</v>
       </c>
+      <c r="D109" s="2"/>
       <c r="E109" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="F109" s="2"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
@@ -2869,9 +2871,11 @@
       <c r="C110" s="3" t="s">
         <v>238</v>
       </c>
+      <c r="D110" s="2"/>
       <c r="E110" s="3" t="s">
         <v>18</v>
       </c>
+      <c r="F110" s="2"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="2">
@@ -2883,9 +2887,11 @@
       <c r="C111" s="3" t="s">
         <v>239</v>
       </c>
+      <c r="D111" s="2"/>
       <c r="E111" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="F111" s="2"/>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
@@ -2897,9 +2903,11 @@
       <c r="C112" s="3" t="s">
         <v>237</v>
       </c>
+      <c r="D112" s="2"/>
       <c r="E112" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="F112" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
basic primary-high schooling system
+ pretty major behind-the-scenes improvements
</commit_message>
<xml_diff>
--- a/assets/achievements/achievements guide.xlsx
+++ b/assets/achievements/achievements guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itsmy\Downloads\bad life simulator\assets\achievements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B84756C-B8F3-49FA-B71F-0362BBBB7B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEDB24E0-D116-4BAE-8077-14F4E2FF2BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="246">
   <si>
     <t>ID</t>
   </si>
@@ -751,6 +751,18 @@
   </si>
   <si>
     <t>Die while committing a murder</t>
+  </si>
+  <si>
+    <t>Integer overflow</t>
+  </si>
+  <si>
+    <t>Incur so much debt that it wraps back around to being positive</t>
+  </si>
+  <si>
+    <t>PhD in subtraction</t>
+  </si>
+  <si>
+    <t>Graduate primary school</t>
   </si>
 </sst>
 </file>
@@ -1086,7 +1098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F114"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.44140625" customWidth="1"/>
@@ -2932,8 +2944,36 @@
       <c r="F113" s="2"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B114" s="3"/>
-      <c r="C114" s="3"/>
+      <c r="A114" s="2">
+        <v>112</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D114" s="2"/>
+      <c r="E114" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F114" s="2"/>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" s="2">
+        <v>113</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D115" s="2"/>
+      <c r="E115" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F115" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>